<commit_message>
Updated on 6th Aug 2026
</commit_message>
<xml_diff>
--- a/Data.xlsx
+++ b/Data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kyndryl-my.sharepoint.com/personal/rohanaggarwal_kyndryl_com1/Documents/Desktop/Temp/Analysis/4Jun2026/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kyndryl-my.sharepoint.com/personal/rohanaggarwal_kyndryl_com1/Documents/Desktop/Temp/Analysis/Github/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_F25DC773A252ABDACC104873E99D53705ADE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{22F9A481-4A05-4733-8BFA-D1BEE8470CD3}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_F25DC773A252ABDACC104873E99D53705ADE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{87F646CD-E5AA-4348-9A5D-4A530B3C277C}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+  <si>
+    <t>Test-6th Aug</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -343,7 +347,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>